<commit_message>
Add FA + Member Federation logo rail to landing page hero
</commit_message>
<xml_diff>
--- a/public/CODA_Course_Candidate_Sheet_Template.xlsx
+++ b/public/CODA_Course_Candidate_Sheet_Template.xlsx
@@ -30,7 +30,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -490,196 +490,342 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:AJ27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="11" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Club</t>
+          <t>Username</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>FA Number</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>External System Id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Courses</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Phone Number</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Date of Birth</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Suborganisation</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Course #</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>SESSION TOPIC 1</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SESSION TOPIC 2</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SESSION TOPIC 3</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SESSION TOPIC 4</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>CET</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Session Topic 1</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Session Topic 2</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Session Topic 3</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Session Topic 4</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (1)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (2)</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (3)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (4)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (5)</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (6)</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (7)</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (8)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>DD/MM/YY (9)</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Goalscoring Presentation</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Annual Plan</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Game Plan</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>4 x Session Plans</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Analysis Session</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Team Meeting / Session Plan</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>6 Week Cycles</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Online Modules</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (1)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (2)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (3)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (4)</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (5)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (6)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (7)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (8)</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>01/01/2026 (9)</t>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>IDP Submitted</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Candidate #</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Jordan Smith</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>1234567</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>jordan.smith@example.com</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
           <t>Northern Suns FC</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>1234567</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Dribbling</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Finishing</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Passing</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Receiving</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Alex Nguyen</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Dribbling</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Finishing</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Passing</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Receiving</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>205</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="V2" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
+      <c r="W2" s="3" t="inlineStr"/>
+      <c r="X2" s="3" t="inlineStr"/>
+      <c r="Y2" s="3" t="inlineStr"/>
+      <c r="Z2" s="3" t="inlineStr"/>
+      <c r="AA2" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AB2" s="3" t="inlineStr"/>
+      <c r="AC2" s="3" t="inlineStr"/>
+      <c r="AD2" s="3" t="inlineStr"/>
+      <c r="AE2" s="3" t="inlineStr"/>
+      <c r="AF2" s="3" t="inlineStr"/>
+      <c r="AG2" s="3" t="inlineStr"/>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="AI2" s="3" t="inlineStr"/>
+      <c r="AJ2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr"/>
@@ -700,6 +846,24 @@
       <c r="P3" s="4" t="inlineStr"/>
       <c r="Q3" s="4" t="inlineStr"/>
       <c r="R3" s="4" t="inlineStr"/>
+      <c r="S3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr"/>
+      <c r="U3" s="4" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr"/>
+      <c r="W3" s="4" t="inlineStr"/>
+      <c r="X3" s="4" t="inlineStr"/>
+      <c r="Y3" s="4" t="inlineStr"/>
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="4" t="inlineStr"/>
+      <c r="AB3" s="4" t="inlineStr"/>
+      <c r="AC3" s="4" t="inlineStr"/>
+      <c r="AD3" s="4" t="inlineStr"/>
+      <c r="AE3" s="4" t="inlineStr"/>
+      <c r="AF3" s="4" t="inlineStr"/>
+      <c r="AG3" s="4" t="inlineStr"/>
+      <c r="AH3" s="4" t="inlineStr"/>
+      <c r="AI3" s="4" t="inlineStr"/>
+      <c r="AJ3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr"/>
@@ -720,6 +884,24 @@
       <c r="P4" s="4" t="inlineStr"/>
       <c r="Q4" s="4" t="inlineStr"/>
       <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr"/>
+      <c r="U4" s="4" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr"/>
+      <c r="W4" s="4" t="inlineStr"/>
+      <c r="X4" s="4" t="inlineStr"/>
+      <c r="Y4" s="4" t="inlineStr"/>
+      <c r="Z4" s="4" t="inlineStr"/>
+      <c r="AA4" s="4" t="inlineStr"/>
+      <c r="AB4" s="4" t="inlineStr"/>
+      <c r="AC4" s="4" t="inlineStr"/>
+      <c r="AD4" s="4" t="inlineStr"/>
+      <c r="AE4" s="4" t="inlineStr"/>
+      <c r="AF4" s="4" t="inlineStr"/>
+      <c r="AG4" s="4" t="inlineStr"/>
+      <c r="AH4" s="4" t="inlineStr"/>
+      <c r="AI4" s="4" t="inlineStr"/>
+      <c r="AJ4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr"/>
@@ -740,6 +922,24 @@
       <c r="P5" s="4" t="inlineStr"/>
       <c r="Q5" s="4" t="inlineStr"/>
       <c r="R5" s="4" t="inlineStr"/>
+      <c r="S5" s="4" t="inlineStr"/>
+      <c r="T5" s="4" t="inlineStr"/>
+      <c r="U5" s="4" t="inlineStr"/>
+      <c r="V5" s="4" t="inlineStr"/>
+      <c r="W5" s="4" t="inlineStr"/>
+      <c r="X5" s="4" t="inlineStr"/>
+      <c r="Y5" s="4" t="inlineStr"/>
+      <c r="Z5" s="4" t="inlineStr"/>
+      <c r="AA5" s="4" t="inlineStr"/>
+      <c r="AB5" s="4" t="inlineStr"/>
+      <c r="AC5" s="4" t="inlineStr"/>
+      <c r="AD5" s="4" t="inlineStr"/>
+      <c r="AE5" s="4" t="inlineStr"/>
+      <c r="AF5" s="4" t="inlineStr"/>
+      <c r="AG5" s="4" t="inlineStr"/>
+      <c r="AH5" s="4" t="inlineStr"/>
+      <c r="AI5" s="4" t="inlineStr"/>
+      <c r="AJ5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr"/>
@@ -760,6 +960,24 @@
       <c r="P6" s="4" t="inlineStr"/>
       <c r="Q6" s="4" t="inlineStr"/>
       <c r="R6" s="4" t="inlineStr"/>
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr"/>
+      <c r="U6" s="4" t="inlineStr"/>
+      <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr"/>
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="4" t="inlineStr"/>
+      <c r="Z6" s="4" t="inlineStr"/>
+      <c r="AA6" s="4" t="inlineStr"/>
+      <c r="AB6" s="4" t="inlineStr"/>
+      <c r="AC6" s="4" t="inlineStr"/>
+      <c r="AD6" s="4" t="inlineStr"/>
+      <c r="AE6" s="4" t="inlineStr"/>
+      <c r="AF6" s="4" t="inlineStr"/>
+      <c r="AG6" s="4" t="inlineStr"/>
+      <c r="AH6" s="4" t="inlineStr"/>
+      <c r="AI6" s="4" t="inlineStr"/>
+      <c r="AJ6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr"/>
@@ -780,6 +998,24 @@
       <c r="P7" s="4" t="inlineStr"/>
       <c r="Q7" s="4" t="inlineStr"/>
       <c r="R7" s="4" t="inlineStr"/>
+      <c r="S7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr"/>
+      <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="inlineStr"/>
+      <c r="X7" s="4" t="inlineStr"/>
+      <c r="Y7" s="4" t="inlineStr"/>
+      <c r="Z7" s="4" t="inlineStr"/>
+      <c r="AA7" s="4" t="inlineStr"/>
+      <c r="AB7" s="4" t="inlineStr"/>
+      <c r="AC7" s="4" t="inlineStr"/>
+      <c r="AD7" s="4" t="inlineStr"/>
+      <c r="AE7" s="4" t="inlineStr"/>
+      <c r="AF7" s="4" t="inlineStr"/>
+      <c r="AG7" s="4" t="inlineStr"/>
+      <c r="AH7" s="4" t="inlineStr"/>
+      <c r="AI7" s="4" t="inlineStr"/>
+      <c r="AJ7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr"/>
@@ -800,6 +1036,24 @@
       <c r="P8" s="4" t="inlineStr"/>
       <c r="Q8" s="4" t="inlineStr"/>
       <c r="R8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr"/>
+      <c r="U8" s="4" t="inlineStr"/>
+      <c r="V8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr"/>
+      <c r="X8" s="4" t="inlineStr"/>
+      <c r="Y8" s="4" t="inlineStr"/>
+      <c r="Z8" s="4" t="inlineStr"/>
+      <c r="AA8" s="4" t="inlineStr"/>
+      <c r="AB8" s="4" t="inlineStr"/>
+      <c r="AC8" s="4" t="inlineStr"/>
+      <c r="AD8" s="4" t="inlineStr"/>
+      <c r="AE8" s="4" t="inlineStr"/>
+      <c r="AF8" s="4" t="inlineStr"/>
+      <c r="AG8" s="4" t="inlineStr"/>
+      <c r="AH8" s="4" t="inlineStr"/>
+      <c r="AI8" s="4" t="inlineStr"/>
+      <c r="AJ8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr"/>
@@ -820,6 +1074,24 @@
       <c r="P9" s="4" t="inlineStr"/>
       <c r="Q9" s="4" t="inlineStr"/>
       <c r="R9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr"/>
+      <c r="U9" s="4" t="inlineStr"/>
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr"/>
+      <c r="X9" s="4" t="inlineStr"/>
+      <c r="Y9" s="4" t="inlineStr"/>
+      <c r="Z9" s="4" t="inlineStr"/>
+      <c r="AA9" s="4" t="inlineStr"/>
+      <c r="AB9" s="4" t="inlineStr"/>
+      <c r="AC9" s="4" t="inlineStr"/>
+      <c r="AD9" s="4" t="inlineStr"/>
+      <c r="AE9" s="4" t="inlineStr"/>
+      <c r="AF9" s="4" t="inlineStr"/>
+      <c r="AG9" s="4" t="inlineStr"/>
+      <c r="AH9" s="4" t="inlineStr"/>
+      <c r="AI9" s="4" t="inlineStr"/>
+      <c r="AJ9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr"/>
@@ -840,6 +1112,24 @@
       <c r="P10" s="4" t="inlineStr"/>
       <c r="Q10" s="4" t="inlineStr"/>
       <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="inlineStr"/>
+      <c r="U10" s="4" t="inlineStr"/>
+      <c r="V10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="inlineStr"/>
+      <c r="X10" s="4" t="inlineStr"/>
+      <c r="Y10" s="4" t="inlineStr"/>
+      <c r="Z10" s="4" t="inlineStr"/>
+      <c r="AA10" s="4" t="inlineStr"/>
+      <c r="AB10" s="4" t="inlineStr"/>
+      <c r="AC10" s="4" t="inlineStr"/>
+      <c r="AD10" s="4" t="inlineStr"/>
+      <c r="AE10" s="4" t="inlineStr"/>
+      <c r="AF10" s="4" t="inlineStr"/>
+      <c r="AG10" s="4" t="inlineStr"/>
+      <c r="AH10" s="4" t="inlineStr"/>
+      <c r="AI10" s="4" t="inlineStr"/>
+      <c r="AJ10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr"/>
@@ -860,6 +1150,24 @@
       <c r="P11" s="4" t="inlineStr"/>
       <c r="Q11" s="4" t="inlineStr"/>
       <c r="R11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr"/>
+      <c r="T11" s="4" t="inlineStr"/>
+      <c r="U11" s="4" t="inlineStr"/>
+      <c r="V11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="inlineStr"/>
+      <c r="X11" s="4" t="inlineStr"/>
+      <c r="Y11" s="4" t="inlineStr"/>
+      <c r="Z11" s="4" t="inlineStr"/>
+      <c r="AA11" s="4" t="inlineStr"/>
+      <c r="AB11" s="4" t="inlineStr"/>
+      <c r="AC11" s="4" t="inlineStr"/>
+      <c r="AD11" s="4" t="inlineStr"/>
+      <c r="AE11" s="4" t="inlineStr"/>
+      <c r="AF11" s="4" t="inlineStr"/>
+      <c r="AG11" s="4" t="inlineStr"/>
+      <c r="AH11" s="4" t="inlineStr"/>
+      <c r="AI11" s="4" t="inlineStr"/>
+      <c r="AJ11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr"/>
@@ -880,6 +1188,24 @@
       <c r="P12" s="4" t="inlineStr"/>
       <c r="Q12" s="4" t="inlineStr"/>
       <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr"/>
+      <c r="U12" s="4" t="inlineStr"/>
+      <c r="V12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="inlineStr"/>
+      <c r="X12" s="4" t="inlineStr"/>
+      <c r="Y12" s="4" t="inlineStr"/>
+      <c r="Z12" s="4" t="inlineStr"/>
+      <c r="AA12" s="4" t="inlineStr"/>
+      <c r="AB12" s="4" t="inlineStr"/>
+      <c r="AC12" s="4" t="inlineStr"/>
+      <c r="AD12" s="4" t="inlineStr"/>
+      <c r="AE12" s="4" t="inlineStr"/>
+      <c r="AF12" s="4" t="inlineStr"/>
+      <c r="AG12" s="4" t="inlineStr"/>
+      <c r="AH12" s="4" t="inlineStr"/>
+      <c r="AI12" s="4" t="inlineStr"/>
+      <c r="AJ12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr"/>
@@ -900,6 +1226,24 @@
       <c r="P13" s="4" t="inlineStr"/>
       <c r="Q13" s="4" t="inlineStr"/>
       <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr"/>
+      <c r="U13" s="4" t="inlineStr"/>
+      <c r="V13" s="4" t="inlineStr"/>
+      <c r="W13" s="4" t="inlineStr"/>
+      <c r="X13" s="4" t="inlineStr"/>
+      <c r="Y13" s="4" t="inlineStr"/>
+      <c r="Z13" s="4" t="inlineStr"/>
+      <c r="AA13" s="4" t="inlineStr"/>
+      <c r="AB13" s="4" t="inlineStr"/>
+      <c r="AC13" s="4" t="inlineStr"/>
+      <c r="AD13" s="4" t="inlineStr"/>
+      <c r="AE13" s="4" t="inlineStr"/>
+      <c r="AF13" s="4" t="inlineStr"/>
+      <c r="AG13" s="4" t="inlineStr"/>
+      <c r="AH13" s="4" t="inlineStr"/>
+      <c r="AI13" s="4" t="inlineStr"/>
+      <c r="AJ13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr"/>
@@ -920,6 +1264,24 @@
       <c r="P14" s="4" t="inlineStr"/>
       <c r="Q14" s="4" t="inlineStr"/>
       <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr"/>
+      <c r="U14" s="4" t="inlineStr"/>
+      <c r="V14" s="4" t="inlineStr"/>
+      <c r="W14" s="4" t="inlineStr"/>
+      <c r="X14" s="4" t="inlineStr"/>
+      <c r="Y14" s="4" t="inlineStr"/>
+      <c r="Z14" s="4" t="inlineStr"/>
+      <c r="AA14" s="4" t="inlineStr"/>
+      <c r="AB14" s="4" t="inlineStr"/>
+      <c r="AC14" s="4" t="inlineStr"/>
+      <c r="AD14" s="4" t="inlineStr"/>
+      <c r="AE14" s="4" t="inlineStr"/>
+      <c r="AF14" s="4" t="inlineStr"/>
+      <c r="AG14" s="4" t="inlineStr"/>
+      <c r="AH14" s="4" t="inlineStr"/>
+      <c r="AI14" s="4" t="inlineStr"/>
+      <c r="AJ14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr"/>
@@ -940,6 +1302,24 @@
       <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr"/>
       <c r="R15" s="4" t="inlineStr"/>
+      <c r="S15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr"/>
+      <c r="U15" s="4" t="inlineStr"/>
+      <c r="V15" s="4" t="inlineStr"/>
+      <c r="W15" s="4" t="inlineStr"/>
+      <c r="X15" s="4" t="inlineStr"/>
+      <c r="Y15" s="4" t="inlineStr"/>
+      <c r="Z15" s="4" t="inlineStr"/>
+      <c r="AA15" s="4" t="inlineStr"/>
+      <c r="AB15" s="4" t="inlineStr"/>
+      <c r="AC15" s="4" t="inlineStr"/>
+      <c r="AD15" s="4" t="inlineStr"/>
+      <c r="AE15" s="4" t="inlineStr"/>
+      <c r="AF15" s="4" t="inlineStr"/>
+      <c r="AG15" s="4" t="inlineStr"/>
+      <c r="AH15" s="4" t="inlineStr"/>
+      <c r="AI15" s="4" t="inlineStr"/>
+      <c r="AJ15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr"/>
@@ -960,6 +1340,24 @@
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
       <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr"/>
+      <c r="U16" s="4" t="inlineStr"/>
+      <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="inlineStr"/>
+      <c r="X16" s="4" t="inlineStr"/>
+      <c r="Y16" s="4" t="inlineStr"/>
+      <c r="Z16" s="4" t="inlineStr"/>
+      <c r="AA16" s="4" t="inlineStr"/>
+      <c r="AB16" s="4" t="inlineStr"/>
+      <c r="AC16" s="4" t="inlineStr"/>
+      <c r="AD16" s="4" t="inlineStr"/>
+      <c r="AE16" s="4" t="inlineStr"/>
+      <c r="AF16" s="4" t="inlineStr"/>
+      <c r="AG16" s="4" t="inlineStr"/>
+      <c r="AH16" s="4" t="inlineStr"/>
+      <c r="AI16" s="4" t="inlineStr"/>
+      <c r="AJ16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr"/>
@@ -980,6 +1378,24 @@
       <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr"/>
       <c r="R17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr"/>
+      <c r="U17" s="4" t="inlineStr"/>
+      <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="inlineStr"/>
+      <c r="X17" s="4" t="inlineStr"/>
+      <c r="Y17" s="4" t="inlineStr"/>
+      <c r="Z17" s="4" t="inlineStr"/>
+      <c r="AA17" s="4" t="inlineStr"/>
+      <c r="AB17" s="4" t="inlineStr"/>
+      <c r="AC17" s="4" t="inlineStr"/>
+      <c r="AD17" s="4" t="inlineStr"/>
+      <c r="AE17" s="4" t="inlineStr"/>
+      <c r="AF17" s="4" t="inlineStr"/>
+      <c r="AG17" s="4" t="inlineStr"/>
+      <c r="AH17" s="4" t="inlineStr"/>
+      <c r="AI17" s="4" t="inlineStr"/>
+      <c r="AJ17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr"/>
@@ -1000,6 +1416,24 @@
       <c r="P18" s="4" t="inlineStr"/>
       <c r="Q18" s="4" t="inlineStr"/>
       <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr"/>
+      <c r="U18" s="4" t="inlineStr"/>
+      <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="inlineStr"/>
+      <c r="X18" s="4" t="inlineStr"/>
+      <c r="Y18" s="4" t="inlineStr"/>
+      <c r="Z18" s="4" t="inlineStr"/>
+      <c r="AA18" s="4" t="inlineStr"/>
+      <c r="AB18" s="4" t="inlineStr"/>
+      <c r="AC18" s="4" t="inlineStr"/>
+      <c r="AD18" s="4" t="inlineStr"/>
+      <c r="AE18" s="4" t="inlineStr"/>
+      <c r="AF18" s="4" t="inlineStr"/>
+      <c r="AG18" s="4" t="inlineStr"/>
+      <c r="AH18" s="4" t="inlineStr"/>
+      <c r="AI18" s="4" t="inlineStr"/>
+      <c r="AJ18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr"/>
@@ -1020,6 +1454,24 @@
       <c r="P19" s="4" t="inlineStr"/>
       <c r="Q19" s="4" t="inlineStr"/>
       <c r="R19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr"/>
+      <c r="U19" s="4" t="inlineStr"/>
+      <c r="V19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr"/>
+      <c r="X19" s="4" t="inlineStr"/>
+      <c r="Y19" s="4" t="inlineStr"/>
+      <c r="Z19" s="4" t="inlineStr"/>
+      <c r="AA19" s="4" t="inlineStr"/>
+      <c r="AB19" s="4" t="inlineStr"/>
+      <c r="AC19" s="4" t="inlineStr"/>
+      <c r="AD19" s="4" t="inlineStr"/>
+      <c r="AE19" s="4" t="inlineStr"/>
+      <c r="AF19" s="4" t="inlineStr"/>
+      <c r="AG19" s="4" t="inlineStr"/>
+      <c r="AH19" s="4" t="inlineStr"/>
+      <c r="AI19" s="4" t="inlineStr"/>
+      <c r="AJ19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr"/>
@@ -1040,6 +1492,24 @@
       <c r="P20" s="4" t="inlineStr"/>
       <c r="Q20" s="4" t="inlineStr"/>
       <c r="R20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr"/>
+      <c r="U20" s="4" t="inlineStr"/>
+      <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr"/>
+      <c r="X20" s="4" t="inlineStr"/>
+      <c r="Y20" s="4" t="inlineStr"/>
+      <c r="Z20" s="4" t="inlineStr"/>
+      <c r="AA20" s="4" t="inlineStr"/>
+      <c r="AB20" s="4" t="inlineStr"/>
+      <c r="AC20" s="4" t="inlineStr"/>
+      <c r="AD20" s="4" t="inlineStr"/>
+      <c r="AE20" s="4" t="inlineStr"/>
+      <c r="AF20" s="4" t="inlineStr"/>
+      <c r="AG20" s="4" t="inlineStr"/>
+      <c r="AH20" s="4" t="inlineStr"/>
+      <c r="AI20" s="4" t="inlineStr"/>
+      <c r="AJ20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr"/>
@@ -1060,6 +1530,24 @@
       <c r="P21" s="4" t="inlineStr"/>
       <c r="Q21" s="4" t="inlineStr"/>
       <c r="R21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr"/>
+      <c r="T21" s="4" t="inlineStr"/>
+      <c r="U21" s="4" t="inlineStr"/>
+      <c r="V21" s="4" t="inlineStr"/>
+      <c r="W21" s="4" t="inlineStr"/>
+      <c r="X21" s="4" t="inlineStr"/>
+      <c r="Y21" s="4" t="inlineStr"/>
+      <c r="Z21" s="4" t="inlineStr"/>
+      <c r="AA21" s="4" t="inlineStr"/>
+      <c r="AB21" s="4" t="inlineStr"/>
+      <c r="AC21" s="4" t="inlineStr"/>
+      <c r="AD21" s="4" t="inlineStr"/>
+      <c r="AE21" s="4" t="inlineStr"/>
+      <c r="AF21" s="4" t="inlineStr"/>
+      <c r="AG21" s="4" t="inlineStr"/>
+      <c r="AH21" s="4" t="inlineStr"/>
+      <c r="AI21" s="4" t="inlineStr"/>
+      <c r="AJ21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr"/>
@@ -1080,6 +1568,214 @@
       <c r="P22" s="4" t="inlineStr"/>
       <c r="Q22" s="4" t="inlineStr"/>
       <c r="R22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr"/>
+      <c r="U22" s="4" t="inlineStr"/>
+      <c r="V22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="inlineStr"/>
+      <c r="X22" s="4" t="inlineStr"/>
+      <c r="Y22" s="4" t="inlineStr"/>
+      <c r="Z22" s="4" t="inlineStr"/>
+      <c r="AA22" s="4" t="inlineStr"/>
+      <c r="AB22" s="4" t="inlineStr"/>
+      <c r="AC22" s="4" t="inlineStr"/>
+      <c r="AD22" s="4" t="inlineStr"/>
+      <c r="AE22" s="4" t="inlineStr"/>
+      <c r="AF22" s="4" t="inlineStr"/>
+      <c r="AG22" s="4" t="inlineStr"/>
+      <c r="AH22" s="4" t="inlineStr"/>
+      <c r="AI22" s="4" t="inlineStr"/>
+      <c r="AJ22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr"/>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
+      <c r="Q23" s="4" t="inlineStr"/>
+      <c r="R23" s="4" t="inlineStr"/>
+      <c r="S23" s="4" t="inlineStr"/>
+      <c r="T23" s="4" t="inlineStr"/>
+      <c r="U23" s="4" t="inlineStr"/>
+      <c r="V23" s="4" t="inlineStr"/>
+      <c r="W23" s="4" t="inlineStr"/>
+      <c r="X23" s="4" t="inlineStr"/>
+      <c r="Y23" s="4" t="inlineStr"/>
+      <c r="Z23" s="4" t="inlineStr"/>
+      <c r="AA23" s="4" t="inlineStr"/>
+      <c r="AB23" s="4" t="inlineStr"/>
+      <c r="AC23" s="4" t="inlineStr"/>
+      <c r="AD23" s="4" t="inlineStr"/>
+      <c r="AE23" s="4" t="inlineStr"/>
+      <c r="AF23" s="4" t="inlineStr"/>
+      <c r="AG23" s="4" t="inlineStr"/>
+      <c r="AH23" s="4" t="inlineStr"/>
+      <c r="AI23" s="4" t="inlineStr"/>
+      <c r="AJ23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="4" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr"/>
+      <c r="O24" s="4" t="inlineStr"/>
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr"/>
+      <c r="U24" s="4" t="inlineStr"/>
+      <c r="V24" s="4" t="inlineStr"/>
+      <c r="W24" s="4" t="inlineStr"/>
+      <c r="X24" s="4" t="inlineStr"/>
+      <c r="Y24" s="4" t="inlineStr"/>
+      <c r="Z24" s="4" t="inlineStr"/>
+      <c r="AA24" s="4" t="inlineStr"/>
+      <c r="AB24" s="4" t="inlineStr"/>
+      <c r="AC24" s="4" t="inlineStr"/>
+      <c r="AD24" s="4" t="inlineStr"/>
+      <c r="AE24" s="4" t="inlineStr"/>
+      <c r="AF24" s="4" t="inlineStr"/>
+      <c r="AG24" s="4" t="inlineStr"/>
+      <c r="AH24" s="4" t="inlineStr"/>
+      <c r="AI24" s="4" t="inlineStr"/>
+      <c r="AJ24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" s="4" t="inlineStr"/>
+      <c r="O25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="inlineStr"/>
+      <c r="Q25" s="4" t="inlineStr"/>
+      <c r="R25" s="4" t="inlineStr"/>
+      <c r="S25" s="4" t="inlineStr"/>
+      <c r="T25" s="4" t="inlineStr"/>
+      <c r="U25" s="4" t="inlineStr"/>
+      <c r="V25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="inlineStr"/>
+      <c r="X25" s="4" t="inlineStr"/>
+      <c r="Y25" s="4" t="inlineStr"/>
+      <c r="Z25" s="4" t="inlineStr"/>
+      <c r="AA25" s="4" t="inlineStr"/>
+      <c r="AB25" s="4" t="inlineStr"/>
+      <c r="AC25" s="4" t="inlineStr"/>
+      <c r="AD25" s="4" t="inlineStr"/>
+      <c r="AE25" s="4" t="inlineStr"/>
+      <c r="AF25" s="4" t="inlineStr"/>
+      <c r="AG25" s="4" t="inlineStr"/>
+      <c r="AH25" s="4" t="inlineStr"/>
+      <c r="AI25" s="4" t="inlineStr"/>
+      <c r="AJ25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr"/>
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr"/>
+      <c r="N26" s="4" t="inlineStr"/>
+      <c r="O26" s="4" t="inlineStr"/>
+      <c r="P26" s="4" t="inlineStr"/>
+      <c r="Q26" s="4" t="inlineStr"/>
+      <c r="R26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr"/>
+      <c r="T26" s="4" t="inlineStr"/>
+      <c r="U26" s="4" t="inlineStr"/>
+      <c r="V26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="inlineStr"/>
+      <c r="X26" s="4" t="inlineStr"/>
+      <c r="Y26" s="4" t="inlineStr"/>
+      <c r="Z26" s="4" t="inlineStr"/>
+      <c r="AA26" s="4" t="inlineStr"/>
+      <c r="AB26" s="4" t="inlineStr"/>
+      <c r="AC26" s="4" t="inlineStr"/>
+      <c r="AD26" s="4" t="inlineStr"/>
+      <c r="AE26" s="4" t="inlineStr"/>
+      <c r="AF26" s="4" t="inlineStr"/>
+      <c r="AG26" s="4" t="inlineStr"/>
+      <c r="AH26" s="4" t="inlineStr"/>
+      <c r="AI26" s="4" t="inlineStr"/>
+      <c r="AJ26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr"/>
+      <c r="O27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr"/>
+      <c r="Q27" s="4" t="inlineStr"/>
+      <c r="R27" s="4" t="inlineStr"/>
+      <c r="S27" s="4" t="inlineStr"/>
+      <c r="T27" s="4" t="inlineStr"/>
+      <c r="U27" s="4" t="inlineStr"/>
+      <c r="V27" s="4" t="inlineStr"/>
+      <c r="W27" s="4" t="inlineStr"/>
+      <c r="X27" s="4" t="inlineStr"/>
+      <c r="Y27" s="4" t="inlineStr"/>
+      <c r="Z27" s="4" t="inlineStr"/>
+      <c r="AA27" s="4" t="inlineStr"/>
+      <c r="AB27" s="4" t="inlineStr"/>
+      <c r="AC27" s="4" t="inlineStr"/>
+      <c r="AD27" s="4" t="inlineStr"/>
+      <c r="AE27" s="4" t="inlineStr"/>
+      <c r="AF27" s="4" t="inlineStr"/>
+      <c r="AG27" s="4" t="inlineStr"/>
+      <c r="AH27" s="4" t="inlineStr"/>
+      <c r="AI27" s="4" t="inlineStr"/>
+      <c r="AJ27" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1108,84 +1804,84 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Fill in the Candidates sheet for the coaches on a course, then upload it via Completed Tasks → Import Coursework CSV in CODA. Save as .csv before uploading (File → Save As → CSV).</t>
+          <t>This matches the column format exported directly from Football Australia's registration system for a course roster. If you export a candidate list from that system, you can rename it and upload it to CODA as-is — no reformatting needed.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Required columns</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Name — required. Used to match against your existing coach roster; anyone not already on file is added automatically.</t>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>To use: fill in (or paste a real export into) the Candidates sheet, save as .csv, then upload it in CODA under Completed Tasks → Import Coursework CSV.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>FA Number — strongly recommended. Used as each coach's unique identifier across CODA.</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Columns CODA actually reads</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>First Name + Last Name — combined automatically into the coach's full name. A coach not already on your CODA roster is added automatically.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Attendance columns (the date columns on the right)</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Username — used as the coach's FA Number in CODA.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Rename each "01/01/2026 (1)" header to the real session date, keeping the bracketed session number — e.g. "12/07/2026 (1)", "19/07/2026 (2)". B Diploma has 9 sessions; C Diploma only needs 4 — delete the columns you don't need.</t>
+          <t>Suborganisation — used as the coach's Club/Team.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Each cell: Y = attended, N (or leave blank) = not attended. You can also use the 3-digit course block code if you have one (starting with 2 for B Diploma, 1 for C Diploma).</t>
+          <t>CET — the tutor assigned to this candidate. Suggested first when starting a New Observation for them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>SESSION TOPIC 1–4 — used for B Diploma only. Leave blank for C Diploma.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Other columns</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>The DD/MM/YY (N) columns — attendance per session. Rename each to the real session date, keeping the bracketed session number, e.g. "12/07/26 (1)". B Diploma has 9 sessions; C Diploma only needs 4 — delete the columns you don't need. Each cell: Y = attended, N or blank = not attended, or a 3-digit block code if you have one (starting with 2 for B Diploma, 1 for C Diploma).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Club — the coach's club or team.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>CET — the tutor assigned to this candidate. CODA will suggest this CET first when starting a New Observation for them.</t>
+          <t>Online Modules — a percentage (e.g. 75), a fraction (e.g. 3/4), or Y/N. Needs to reach 100% to count as complete.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Session Topic 1–4 — only used for B Diploma. Leave blank for C Diploma (Session Activity is set per-observation instead).</t>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Columns kept for reference but not currently read by CODA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Online Modules — a percentage (e.g. 75), a fraction (e.g. 3/4), or Y/N. Needs to reach 100% to count as complete.</t>
+          <t>Status, External System Id, Courses, Email, Phone Number, Date of Birth, Department, Course #, Goalscoring Presentation, Annual Plan, Game Plan, 4 x Session Plans, Analysis Session, Team Meeting / Session Plan, 6 Week Cycles, IDP Submitted, Candidate # — these import fine (they're just ignored), so a real export can be uploaded unedited. The individual coursework milestones (Annual Plan, Game Plan, etc.) are tracked inside CODA itself, one tick at a time, as each is completed — Course Number is entered separately in CODA's upload screen, not read from this sheet.</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1895,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>In CODA, go to Completed Tasks → Import Coursework CSV, choose B or C Diploma, and enter the Course Title and Course Number for this course — Course Number is required.</t>
+          <t>In CODA, go to Completed Tasks → Import Coursework CSV, choose B or C Diploma, and enter the Course Title and Course Number — Course Number is required.</t>
         </is>
       </c>
     </row>

</xml_diff>